<commit_message>
error en rodll linea lana
</commit_message>
<xml_diff>
--- a/LISTAS/ma/ARANDELA CHAPISTA y comunes.xlsx
+++ b/LISTAS/ma/ARANDELA CHAPISTA y comunes.xlsx
@@ -899,16 +899,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="19" t="n">
-        <v>45183.57414958789</v>
+        <v>45253</v>
       </c>
       <c r="F1" s="40" t="n"/>
       <c r="G1" s="40" t="n"/>
       <c r="H1" s="41" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="42">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -930,7 +926,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="22.5" customHeight="1" s="42">
       <c r="A10" s="36" t="inlineStr">
         <is>
@@ -948,25 +943,6 @@
       <c r="G11" s="37" t="n"/>
       <c r="H11" s="34" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31" ht="18" customHeight="1" s="42">
       <c r="A31" s="18" t="inlineStr">
         <is>
@@ -1007,7 +983,7 @@
       </c>
       <c r="C33" s="44" t="n"/>
       <c r="D33" s="9" t="n">
-        <v>2988.714</v>
+        <v>3287.585</v>
       </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="42">
@@ -1021,7 +997,7 @@
       </c>
       <c r="C34" s="44" t="n"/>
       <c r="D34" s="9" t="n">
-        <v>2245.542</v>
+        <v>2470.096</v>
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="42">
@@ -1035,7 +1011,7 @@
       </c>
       <c r="C35" s="44" t="n"/>
       <c r="D35" s="9" t="n">
-        <v>1937.783</v>
+        <v>2131.561</v>
       </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="42">
@@ -1049,7 +1025,7 @@
       </c>
       <c r="C36" s="44" t="n"/>
       <c r="D36" s="9" t="n">
-        <v>1740.206</v>
+        <v>1914.227</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="42">
@@ -1063,7 +1039,7 @@
       </c>
       <c r="C37" s="44" t="n"/>
       <c r="D37" s="9" t="n">
-        <v>1740.206</v>
+        <v>1914.227</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="42">
@@ -1077,7 +1053,7 @@
       </c>
       <c r="C38" s="44" t="n"/>
       <c r="D38" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" s="42">
@@ -1091,7 +1067,7 @@
       </c>
       <c r="C39" s="44" t="n"/>
       <c r="D39" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="42">
@@ -1105,7 +1081,7 @@
       </c>
       <c r="C40" s="44" t="n"/>
       <c r="D40" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" s="42">
@@ -1119,7 +1095,7 @@
       </c>
       <c r="C41" s="44" t="n"/>
       <c r="D41" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="42">
@@ -1133,7 +1109,7 @@
       </c>
       <c r="C42" s="44" t="n"/>
       <c r="D42" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="42">
@@ -1147,7 +1123,7 @@
       </c>
       <c r="C43" s="44" t="n"/>
       <c r="D43" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="42">
@@ -1163,7 +1139,7 @@
       </c>
       <c r="C44" s="44" t="n"/>
       <c r="D44" s="9" t="n">
-        <v>1467.771</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="45" ht="16.5" customHeight="1" s="42">
@@ -1179,7 +1155,7 @@
       </c>
       <c r="C45" s="44" t="n"/>
       <c r="D45" s="9" t="n">
-        <v>1751.603</v>
+        <v>1926.763</v>
       </c>
     </row>
     <row r="46" ht="16.5" customHeight="1" s="42">
@@ -1195,7 +1171,7 @@
       </c>
       <c r="C46" s="44" t="n"/>
       <c r="D46" s="9" t="n">
-        <v>1751.603</v>
+        <v>1926.763</v>
       </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="42">
@@ -1211,10 +1187,9 @@
       </c>
       <c r="C47" s="44" t="n"/>
       <c r="D47" s="9" t="n">
-        <v>1751.603</v>
-      </c>
-    </row>
-    <row r="48"/>
+        <v>1926.763</v>
+      </c>
+    </row>
     <row r="49" ht="18" customHeight="1" s="42">
       <c r="A49" s="18" t="inlineStr">
         <is>
@@ -1254,7 +1229,7 @@
       </c>
       <c r="C51" s="44" t="n"/>
       <c r="D51" s="9" t="n">
-        <v>2553.313</v>
+        <v>2808.644</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="42">
@@ -1268,7 +1243,7 @@
       </c>
       <c r="C52" s="44" t="n"/>
       <c r="D52" s="9" t="n">
-        <v>2321.542</v>
+        <v>2553.696</v>
       </c>
     </row>
     <row r="53" ht="23.25" customHeight="1" s="42">
@@ -1282,7 +1257,7 @@
       </c>
       <c r="C53" s="44" t="n"/>
       <c r="D53" s="9" t="n">
-        <v>1937.783</v>
+        <v>2131.561</v>
       </c>
       <c r="E53" s="10" t="n"/>
       <c r="F53" s="10" t="n"/>
@@ -1300,7 +1275,7 @@
       </c>
       <c r="C54" s="44" t="n"/>
       <c r="D54" s="9" t="n">
-        <v>1937.783</v>
+        <v>2131.561</v>
       </c>
       <c r="E54" s="11" t="n"/>
       <c r="F54" s="11" t="n"/>
@@ -1327,7 +1302,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -1335,18 +1309,8 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
     <row r="64" ht="18" customHeight="1" s="42"/>
     <row r="65" ht="18" customHeight="1" s="42"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72" ht="62.25" customHeight="1" s="42"/>
     <row r="73" ht="18" customHeight="1" s="42">
       <c r="C73" s="20" t="n"/>
@@ -1381,37 +1345,37 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D77:E77"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="D73:E73"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B50:C50"/>
     <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="D77:E77"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
corregi lo de q algunos articulso no llevan precios y agregue un boton obtner precios en la vista step1
</commit_message>
<xml_diff>
--- a/LISTAS/ma/ARANDELA CHAPISTA y comunes.xlsx
+++ b/LISTAS/ma/ARANDELA CHAPISTA y comunes.xlsx
@@ -899,12 +899,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="19" t="n">
-        <v>45266</v>
+        <v>45264.54806026705</v>
       </c>
       <c r="F1" s="40" t="n"/>
       <c r="G1" s="40" t="n"/>
       <c r="H1" s="41" t="n"/>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="42">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -926,6 +930,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="22.5" customHeight="1" s="42">
       <c r="A10" s="36" t="inlineStr">
         <is>
@@ -943,6 +948,25 @@
       <c r="G11" s="37" t="n"/>
       <c r="H11" s="34" t="n"/>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31" ht="18" customHeight="1" s="42">
       <c r="A31" s="18" t="inlineStr">
         <is>
@@ -983,7 +1007,7 @@
       </c>
       <c r="C33" s="44" t="n"/>
       <c r="D33" s="9" t="n">
-        <v>3287.585</v>
+        <v>4374.33</v>
       </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="42">
@@ -997,7 +1021,7 @@
       </c>
       <c r="C34" s="44" t="n"/>
       <c r="D34" s="9" t="n">
-        <v>2470.096</v>
+        <v>3286.61</v>
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="42">
@@ -1011,7 +1035,7 @@
       </c>
       <c r="C35" s="44" t="n"/>
       <c r="D35" s="9" t="n">
-        <v>2131.561</v>
+        <v>2836.16</v>
       </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="42">
@@ -1025,7 +1049,7 @@
       </c>
       <c r="C36" s="44" t="n"/>
       <c r="D36" s="9" t="n">
-        <v>1914.227</v>
+        <v>2546.99</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="42">
@@ -1039,7 +1063,7 @@
       </c>
       <c r="C37" s="44" t="n"/>
       <c r="D37" s="9" t="n">
-        <v>1914.227</v>
+        <v>2546.99</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="42">
@@ -1053,7 +1077,7 @@
       </c>
       <c r="C38" s="44" t="n"/>
       <c r="D38" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" s="42">
@@ -1067,7 +1091,7 @@
       </c>
       <c r="C39" s="44" t="n"/>
       <c r="D39" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="42">
@@ -1081,7 +1105,7 @@
       </c>
       <c r="C40" s="44" t="n"/>
       <c r="D40" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" s="42">
@@ -1095,7 +1119,7 @@
       </c>
       <c r="C41" s="44" t="n"/>
       <c r="D41" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="42">
@@ -1109,7 +1133,7 @@
       </c>
       <c r="C42" s="44" t="n"/>
       <c r="D42" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="42">
@@ -1123,7 +1147,7 @@
       </c>
       <c r="C43" s="44" t="n"/>
       <c r="D43" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="42">
@@ -1139,7 +1163,7 @@
       </c>
       <c r="C44" s="44" t="n"/>
       <c r="D44" s="9" t="n">
-        <v>1614.548</v>
+        <v>2148.25</v>
       </c>
     </row>
     <row r="45" ht="16.5" customHeight="1" s="42">
@@ -1155,7 +1179,7 @@
       </c>
       <c r="C45" s="44" t="n"/>
       <c r="D45" s="9" t="n">
-        <v>1926.763</v>
+        <v>2563.67</v>
       </c>
     </row>
     <row r="46" ht="16.5" customHeight="1" s="42">
@@ -1171,7 +1195,7 @@
       </c>
       <c r="C46" s="44" t="n"/>
       <c r="D46" s="9" t="n">
-        <v>1926.763</v>
+        <v>2563.67</v>
       </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="42">
@@ -1187,9 +1211,10 @@
       </c>
       <c r="C47" s="44" t="n"/>
       <c r="D47" s="9" t="n">
-        <v>1926.763</v>
-      </c>
-    </row>
+        <v>2563.67</v>
+      </c>
+    </row>
+    <row r="48"/>
     <row r="49" ht="18" customHeight="1" s="42">
       <c r="A49" s="18" t="inlineStr">
         <is>
@@ -1229,7 +1254,7 @@
       </c>
       <c r="C51" s="44" t="n"/>
       <c r="D51" s="9" t="n">
-        <v>2808.644</v>
+        <v>3737.06</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="42">
@@ -1243,7 +1268,7 @@
       </c>
       <c r="C52" s="44" t="n"/>
       <c r="D52" s="9" t="n">
-        <v>2553.696</v>
+        <v>3397.84</v>
       </c>
     </row>
     <row r="53" ht="23.25" customHeight="1" s="42">
@@ -1257,7 +1282,7 @@
       </c>
       <c r="C53" s="44" t="n"/>
       <c r="D53" s="9" t="n">
-        <v>2131.561</v>
+        <v>2836.16</v>
       </c>
       <c r="E53" s="10" t="n"/>
       <c r="F53" s="10" t="n"/>
@@ -1275,7 +1300,7 @@
       </c>
       <c r="C54" s="44" t="n"/>
       <c r="D54" s="9" t="n">
-        <v>2131.561</v>
+        <v>2836.16</v>
       </c>
       <c r="E54" s="11" t="n"/>
       <c r="F54" s="11" t="n"/>
@@ -1302,6 +1327,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -1309,8 +1335,18 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
     <row r="64" ht="18" customHeight="1" s="42"/>
     <row r="65" ht="18" customHeight="1" s="42"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
     <row r="72" ht="62.25" customHeight="1" s="42"/>
     <row r="73" ht="18" customHeight="1" s="42">
       <c r="C73" s="20" t="n"/>
@@ -1345,37 +1381,37 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
     <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D73:E73"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B54:C54"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D77:E77"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="B42:C42"/>
     <mergeCell ref="A49:D49"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
agregue el checkbnox para chekear todo
</commit_message>
<xml_diff>
--- a/LISTAS/ma/ARANDELA CHAPISTA y comunes.xlsx
+++ b/LISTAS/ma/ARANDELA CHAPISTA y comunes.xlsx
@@ -899,16 +899,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="19" t="n">
-        <v>45264.54806026705</v>
+        <v>45286</v>
       </c>
       <c r="F1" s="40" t="n"/>
       <c r="G1" s="40" t="n"/>
       <c r="H1" s="41" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="42">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -930,7 +926,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="22.5" customHeight="1" s="42">
       <c r="A10" s="36" t="inlineStr">
         <is>
@@ -948,25 +943,6 @@
       <c r="G11" s="37" t="n"/>
       <c r="H11" s="34" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31" ht="18" customHeight="1" s="42">
       <c r="A31" s="18" t="inlineStr">
         <is>
@@ -1007,7 +983,7 @@
       </c>
       <c r="C33" s="44" t="n"/>
       <c r="D33" s="9" t="n">
-        <v>4374.33</v>
+        <v>3287.585</v>
       </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="42">
@@ -1021,7 +997,7 @@
       </c>
       <c r="C34" s="44" t="n"/>
       <c r="D34" s="9" t="n">
-        <v>3286.61</v>
+        <v>2470.096</v>
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="42">
@@ -1035,7 +1011,7 @@
       </c>
       <c r="C35" s="44" t="n"/>
       <c r="D35" s="9" t="n">
-        <v>2836.16</v>
+        <v>2131.561</v>
       </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="42">
@@ -1049,7 +1025,7 @@
       </c>
       <c r="C36" s="44" t="n"/>
       <c r="D36" s="9" t="n">
-        <v>2546.99</v>
+        <v>1914.227</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="42">
@@ -1063,7 +1039,7 @@
       </c>
       <c r="C37" s="44" t="n"/>
       <c r="D37" s="9" t="n">
-        <v>2546.99</v>
+        <v>1914.227</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="42">
@@ -1077,7 +1053,7 @@
       </c>
       <c r="C38" s="44" t="n"/>
       <c r="D38" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" s="42">
@@ -1091,7 +1067,7 @@
       </c>
       <c r="C39" s="44" t="n"/>
       <c r="D39" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="42">
@@ -1105,7 +1081,7 @@
       </c>
       <c r="C40" s="44" t="n"/>
       <c r="D40" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" s="42">
@@ -1119,7 +1095,7 @@
       </c>
       <c r="C41" s="44" t="n"/>
       <c r="D41" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="42">
@@ -1133,7 +1109,7 @@
       </c>
       <c r="C42" s="44" t="n"/>
       <c r="D42" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="42">
@@ -1147,7 +1123,7 @@
       </c>
       <c r="C43" s="44" t="n"/>
       <c r="D43" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="42">
@@ -1163,7 +1139,7 @@
       </c>
       <c r="C44" s="44" t="n"/>
       <c r="D44" s="9" t="n">
-        <v>2148.25</v>
+        <v>1614.548</v>
       </c>
     </row>
     <row r="45" ht="16.5" customHeight="1" s="42">
@@ -1179,7 +1155,7 @@
       </c>
       <c r="C45" s="44" t="n"/>
       <c r="D45" s="9" t="n">
-        <v>2563.67</v>
+        <v>1926.763</v>
       </c>
     </row>
     <row r="46" ht="16.5" customHeight="1" s="42">
@@ -1195,7 +1171,7 @@
       </c>
       <c r="C46" s="44" t="n"/>
       <c r="D46" s="9" t="n">
-        <v>2563.67</v>
+        <v>1926.763</v>
       </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="42">
@@ -1211,10 +1187,9 @@
       </c>
       <c r="C47" s="44" t="n"/>
       <c r="D47" s="9" t="n">
-        <v>2563.67</v>
-      </c>
-    </row>
-    <row r="48"/>
+        <v>1926.763</v>
+      </c>
+    </row>
     <row r="49" ht="18" customHeight="1" s="42">
       <c r="A49" s="18" t="inlineStr">
         <is>
@@ -1254,7 +1229,7 @@
       </c>
       <c r="C51" s="44" t="n"/>
       <c r="D51" s="9" t="n">
-        <v>3737.06</v>
+        <v>2808.644</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="42">
@@ -1268,7 +1243,7 @@
       </c>
       <c r="C52" s="44" t="n"/>
       <c r="D52" s="9" t="n">
-        <v>3397.84</v>
+        <v>2553.696</v>
       </c>
     </row>
     <row r="53" ht="23.25" customHeight="1" s="42">
@@ -1282,7 +1257,7 @@
       </c>
       <c r="C53" s="44" t="n"/>
       <c r="D53" s="9" t="n">
-        <v>2836.16</v>
+        <v>2131.561</v>
       </c>
       <c r="E53" s="10" t="n"/>
       <c r="F53" s="10" t="n"/>
@@ -1300,7 +1275,7 @@
       </c>
       <c r="C54" s="44" t="n"/>
       <c r="D54" s="9" t="n">
-        <v>2836.16</v>
+        <v>2131.561</v>
       </c>
       <c r="E54" s="11" t="n"/>
       <c r="F54" s="11" t="n"/>
@@ -1327,7 +1302,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -1335,18 +1309,8 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
     <row r="64" ht="18" customHeight="1" s="42"/>
     <row r="65" ht="18" customHeight="1" s="42"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72" ht="62.25" customHeight="1" s="42"/>
     <row r="73" ht="18" customHeight="1" s="42">
       <c r="C73" s="20" t="n"/>
@@ -1381,37 +1345,37 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D73:E73"/>
     <mergeCell ref="B46:C46"/>
     <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="D75:E75"/>
     <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B44:C44"/>
     <mergeCell ref="D77:E77"/>
     <mergeCell ref="D76:E76"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="D75:E75"/>
     <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="A49:D49"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B51:C51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>